<commit_message>
Add Lead Reports filter cases (LR-147…166) and the traceability matrix
- LR-147…156: filter combinations, clearing a filter, "All" values,
  single-lead and empty results, Unspecified values, tab switching and
  filter master data (filter-combinations.spec.ts)
- LR-157…166: each of the 8 filters applied in turn, with every count on
  every tab checked against the page itself (filter-counts.spec.ts)
- Shared filter helpers in tests/lead-reports/filters.ts
- Rows, results and Summary ranges added to Lead_Reports_Test_Cases.xlsx
- Testcase/Reports_Traceability_Matrix.xlsx: 98 requirements → 599 test
  cases → latest result (16-Oct-2026 run) → defects
- tableColumn waits for the table header before reading (fixes RA-082)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Testcase/Lead_Reports_Test_Cases.xlsx
+++ b/Testcase/Lead_Reports_Test_Cases.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Observations" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$1:$M$147</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$1:$M$167</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Test Cases'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Drill-down Verification'!$A$1:$O$180</definedName>
   </definedNames>
@@ -70,7 +70,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -107,6 +107,11 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -134,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -168,6 +173,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -552,7 +560,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -625,7 +632,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -660,19 +666,19 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Test Cases'!$B$2:$B$147,A11)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$167,A11)</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A11,'Test Cases'!$K$2:$K$147,"High")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A11,'Test Cases'!$K$2:$K$167,"High")</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A11,'Test Cases'!$L$2:$L$147,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A11,'Test Cases'!$L$2:$L$167,"Pass")</f>
         <v/>
       </c>
       <c r="E11" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A11,'Test Cases'!$L$2:$L$147,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A11,'Test Cases'!$L$2:$L$167,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -683,19 +689,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('Test Cases'!$B$2:$B$147,A12)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$167,A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A12,'Test Cases'!$K$2:$K$147,"High")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A12,'Test Cases'!$K$2:$K$167,"High")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A12,'Test Cases'!$L$2:$L$147,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A12,'Test Cases'!$L$2:$L$167,"Pass")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A12,'Test Cases'!$L$2:$L$147,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A12,'Test Cases'!$L$2:$L$167,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -706,19 +712,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('Test Cases'!$B$2:$B$147,A13)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$167,A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A13,'Test Cases'!$K$2:$K$147,"High")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A13,'Test Cases'!$K$2:$K$167,"High")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A13,'Test Cases'!$L$2:$L$147,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A13,'Test Cases'!$L$2:$L$167,"Pass")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A13,'Test Cases'!$L$2:$L$147,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A13,'Test Cases'!$L$2:$L$167,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -729,19 +735,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('Test Cases'!$B$2:$B$147,A14)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$167,A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A14,'Test Cases'!$K$2:$K$147,"High")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A14,'Test Cases'!$K$2:$K$167,"High")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A14,'Test Cases'!$L$2:$L$147,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A14,'Test Cases'!$L$2:$L$167,"Pass")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A14,'Test Cases'!$L$2:$L$147,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A14,'Test Cases'!$L$2:$L$167,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -752,19 +758,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('Test Cases'!$B$2:$B$147,A15)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$167,A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A15,'Test Cases'!$K$2:$K$147,"High")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A15,'Test Cases'!$K$2:$K$167,"High")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A15,'Test Cases'!$L$2:$L$147,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A15,'Test Cases'!$L$2:$L$167,"Pass")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A15,'Test Cases'!$L$2:$L$147,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A15,'Test Cases'!$L$2:$L$167,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -775,19 +781,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('Test Cases'!$B$2:$B$147,A16)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$167,A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A16,'Test Cases'!$K$2:$K$147,"High")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A16,'Test Cases'!$K$2:$K$167,"High")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A16,'Test Cases'!$L$2:$L$147,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A16,'Test Cases'!$L$2:$L$167,"Pass")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A16,'Test Cases'!$L$2:$L$147,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A16,'Test Cases'!$L$2:$L$167,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -798,19 +804,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('Test Cases'!$B$2:$B$147,A17)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$167,A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A17,'Test Cases'!$K$2:$K$147,"High")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A17,'Test Cases'!$K$2:$K$167,"High")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A17,'Test Cases'!$L$2:$L$147,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A17,'Test Cases'!$L$2:$L$167,"Pass")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A17,'Test Cases'!$L$2:$L$147,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A17,'Test Cases'!$L$2:$L$167,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -821,19 +827,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('Test Cases'!$B$2:$B$147,A18)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$167,A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A18,'Test Cases'!$K$2:$K$147,"High")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A18,'Test Cases'!$K$2:$K$167,"High")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A18,'Test Cases'!$L$2:$L$147,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A18,'Test Cases'!$L$2:$L$167,"Pass")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A18,'Test Cases'!$L$2:$L$147,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A18,'Test Cases'!$L$2:$L$167,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -844,19 +850,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('Test Cases'!$B$2:$B$147,A19)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$167,A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A19,'Test Cases'!$K$2:$K$147,"High")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A19,'Test Cases'!$K$2:$K$167,"High")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A19,'Test Cases'!$L$2:$L$147,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A19,'Test Cases'!$L$2:$L$167,"Pass")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A19,'Test Cases'!$L$2:$L$147,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A19,'Test Cases'!$L$2:$L$167,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -867,19 +873,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('Test Cases'!$B$2:$B$147,A20)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$167,A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A20,'Test Cases'!$K$2:$K$147,"High")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A20,'Test Cases'!$K$2:$K$167,"High")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A20,'Test Cases'!$L$2:$L$147,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A20,'Test Cases'!$L$2:$L$167,"Pass")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A20,'Test Cases'!$L$2:$L$147,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A20,'Test Cases'!$L$2:$L$167,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -890,19 +896,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('Test Cases'!$B$2:$B$147,A21)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$167,A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A21,'Test Cases'!$K$2:$K$147,"High")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A21,'Test Cases'!$K$2:$K$167,"High")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A21,'Test Cases'!$L$2:$L$147,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A21,'Test Cases'!$L$2:$L$167,"Pass")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$147,A21,'Test Cases'!$L$2:$L$147,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$167,A21,'Test Cases'!$L$2:$L$167,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -929,7 +935,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
@@ -949,7 +954,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF('Test Cases'!$J$2:$J$147,A25)</f>
+        <f>COUNTIF('Test Cases'!$J$2:$J$167,A25)</f>
         <v/>
       </c>
     </row>
@@ -960,7 +965,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('Test Cases'!$J$2:$J$147,A26)</f>
+        <f>COUNTIF('Test Cases'!$J$2:$J$167,A26)</f>
         <v/>
       </c>
     </row>
@@ -971,7 +976,7 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('Test Cases'!$J$2:$J$147,A27)</f>
+        <f>COUNTIF('Test Cases'!$J$2:$J$167,A27)</f>
         <v/>
       </c>
     </row>
@@ -982,7 +987,7 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('Test Cases'!$J$2:$J$147,A28)</f>
+        <f>COUNTIF('Test Cases'!$J$2:$J$167,A28)</f>
         <v/>
       </c>
     </row>
@@ -993,7 +998,7 @@
         </is>
       </c>
       <c r="B29" s="5">
-        <f>COUNTIF('Test Cases'!$J$2:$J$147,A29)</f>
+        <f>COUNTIF('Test Cases'!$J$2:$J$167,A29)</f>
         <v/>
       </c>
     </row>
@@ -1004,7 +1009,7 @@
         </is>
       </c>
       <c r="B30" s="5">
-        <f>COUNTIF('Test Cases'!$J$2:$J$147,A30)</f>
+        <f>COUNTIF('Test Cases'!$J$2:$J$167,A30)</f>
         <v/>
       </c>
     </row>
@@ -1015,7 +1020,7 @@
         </is>
       </c>
       <c r="B31" s="5">
-        <f>COUNTIF('Test Cases'!$J$2:$J$147,A31)</f>
+        <f>COUNTIF('Test Cases'!$J$2:$J$167,A31)</f>
         <v/>
       </c>
     </row>
@@ -1026,11 +1031,10 @@
         </is>
       </c>
       <c r="B32" s="5">
-        <f>COUNTIF('Test Cases'!$J$2:$J$147,A32)</f>
+        <f>COUNTIF('Test Cases'!$J$2:$J$167,A32)</f>
         <v/>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
@@ -1050,7 +1054,7 @@
         </is>
       </c>
       <c r="B35" s="5">
-        <f>COUNTIF('Test Cases'!$K$2:$K$147,A35)</f>
+        <f>COUNTIF('Test Cases'!$K$2:$K$167,A35)</f>
         <v/>
       </c>
     </row>
@@ -1061,7 +1065,7 @@
         </is>
       </c>
       <c r="B36" s="5">
-        <f>COUNTIF('Test Cases'!$K$2:$K$147,A36)</f>
+        <f>COUNTIF('Test Cases'!$K$2:$K$167,A36)</f>
         <v/>
       </c>
     </row>
@@ -1072,11 +1076,10 @@
         </is>
       </c>
       <c r="B37" s="5">
-        <f>COUNTIF('Test Cases'!$K$2:$K$147,A37)</f>
+        <f>COUNTIF('Test Cases'!$K$2:$K$167,A37)</f>
         <v/>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
@@ -1096,7 +1099,7 @@
         </is>
       </c>
       <c r="B40" s="5">
-        <f>COUNTIF('Test Cases'!$L$2:$L$147,A40)</f>
+        <f>COUNTIF('Test Cases'!$L$2:$L$167,A40)</f>
         <v/>
       </c>
     </row>
@@ -1107,7 +1110,7 @@
         </is>
       </c>
       <c r="B41" s="5">
-        <f>COUNTIF('Test Cases'!$L$2:$L$147,A41)</f>
+        <f>COUNTIF('Test Cases'!$L$2:$L$167,A41)</f>
         <v/>
       </c>
     </row>
@@ -1118,7 +1121,7 @@
         </is>
       </c>
       <c r="B42" s="5">
-        <f>COUNTIF('Test Cases'!$L$2:$L$147,A42)</f>
+        <f>COUNTIF('Test Cases'!$L$2:$L$167,A42)</f>
         <v/>
       </c>
     </row>
@@ -1129,7 +1132,7 @@
         </is>
       </c>
       <c r="B43" s="5">
-        <f>COUNTIF('Test Cases'!$L$2:$L$147,A43)</f>
+        <f>COUNTIF('Test Cases'!$L$2:$L$167,A43)</f>
         <v/>
       </c>
     </row>
@@ -1140,11 +1143,10 @@
         </is>
       </c>
       <c r="B44" s="5">
-        <f>COUNTIF('Test Cases'!$L$2:$L$147,A44)</f>
+        <f>COUNTIF('Test Cases'!$L$2:$L$167,A44)</f>
         <v/>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
@@ -1212,7 +1214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M147"/>
+  <dimension ref="A1:M167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10201,13 +10203,1403 @@
         </is>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" s="8" t="inlineStr">
+        <is>
+          <t>LR-147</t>
+        </is>
+      </c>
+      <c r="B148" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C148" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="D148" s="8" t="inlineStr">
+        <is>
+          <t>Verify All filters together return only records matching every selected filter</t>
+        </is>
+      </c>
+      <c r="E148" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F148" s="8" t="inlineStr">
+        <is>
+          <t>1. Period = Last 12 months
+2. For each filter in turn (Lead Source, Capture Channel, Campaign, Broker, Salesperson, Project, Nationality, Prospect Type): open Source &amp; Channel › Performance by &lt;that field&gt; and pick a value that still has leads under the filters already applied
+3. Apply it in the header filter
+4. After each filter, read Leads Captured</t>
+        </is>
+      </c>
+      <c r="G148" s="8" t="inlineStr">
+        <is>
+          <t>Last 12 months; filter values are picked from the page at run time</t>
+        </is>
+      </c>
+      <c r="H148" s="8" t="inlineStr">
+        <is>
+          <t>After each filter Leads Captured equals the picked row's Leads and never goes up; a field with no remaining value stays at "All"; the final count is the leads matching every selected filter</t>
+        </is>
+      </c>
+      <c r="I148" s="8" t="inlineStr">
+        <is>
+          <t>All 613 → Lead Source Digital Marketing 18 → Capture Channel Google Ads 5 → Campaign Palm Exotica Campaign 2026-01 2 → Salesperson CRM Administrator 2 → Nationality Australia 1 (Broker, Project, Prospect Type had no value left); list = export = 1 lead, matching Source, Channel and Salesperson</t>
+        </is>
+      </c>
+      <c r="J148" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K148" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L148" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M148" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-combinations.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="8" t="inlineStr">
+        <is>
+          <t>LR-148</t>
+        </is>
+      </c>
+      <c r="B149" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C149" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="D149" s="8" t="inlineStr">
+        <is>
+          <t>Verify changing one filter recalculates all KPI cards and report tables</t>
+        </is>
+      </c>
+      <c r="E149" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F149" s="8" t="inlineStr">
+        <is>
+          <t>1. Period = Last 12 months; note every KPI card
+2. Set Lead Source to a source that has some, but not all, leads
+3. Check every KPI card, the Lead Funnel, the Source &amp; Channel Total and the Salesperson Scorecard</t>
+        </is>
+      </c>
+      <c r="G149" s="8" t="inlineStr">
+        <is>
+          <t>Last 12 months; filter values are picked from the page at run time</t>
+        </is>
+      </c>
+      <c r="H149" s="8" t="inlineStr">
+        <is>
+          <t>Leads Captured = that source's row; every count card is ≤ its unfiltered value; Contact / Qualification / Opportunity rates = funnel step ÷ Leads Captured; funnel Captured, Source &amp; Channel Total and Scorecard Leads all equal the new Leads Captured</t>
+        </is>
+      </c>
+      <c r="I149" s="8" t="inlineStr">
+        <is>
+          <t>Lead Source = Digital Marketing: Leads Captured 613 → 18; Contact 52.7% → 77.8%, Qualification 40.9% → 77.8%, Opportunity 20.1% → 66.7% (= subtitle counts ÷ 18); SPA Signed 78 → 7; Open Leads Now 362 → 6; funnel, Source &amp; Channel Total and Scorecard Leads = 18</t>
+        </is>
+      </c>
+      <c r="J149" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K149" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L149" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M149" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-combinations.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="8" t="inlineStr">
+        <is>
+          <t>LR-149</t>
+        </is>
+      </c>
+      <c r="B150" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C150" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="D150" s="8" t="inlineStr">
+        <is>
+          <t>Verify clearing one selected filter restores only that filter's data while retaining other filters</t>
+        </is>
+      </c>
+      <c r="E150" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F150" s="8" t="inlineStr">
+        <is>
+          <t>1. Period = Last 12 months; note Leads Captured for Lead Source = A alone and for Project = P alone
+2. Apply Lead Source = A and Project = P
+3. Set Project back to "All projects"
+4. Set Project = P again, then Lead Source back to "All sources"</t>
+        </is>
+      </c>
+      <c r="G150" s="8" t="inlineStr">
+        <is>
+          <t>Last 12 months; filter values are picked from the page at run time</t>
+        </is>
+      </c>
+      <c r="H150" s="8" t="inlineStr">
+        <is>
+          <t>After step 3 Lead Source is still A and Leads Captured = A alone; after step 4 Project is still P and Leads Captured = P alone</t>
+        </is>
+      </c>
+      <c r="I150" s="8" t="inlineStr">
+        <is>
+          <t>Digital Marketing alone 18, Palm Exotjca Limited alone 555, both 1; clearing Project → 18 with Lead Source kept; clearing Lead Source → 555 with Project kept</t>
+        </is>
+      </c>
+      <c r="J150" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K150" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L150" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M150" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-combinations.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="8" t="inlineStr">
+        <is>
+          <t>LR-150</t>
+        </is>
+      </c>
+      <c r="B151" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C151" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="D151" s="8" t="inlineStr">
+        <is>
+          <t>Verify selecting All for every filter returns the unfiltered report totals</t>
+        </is>
+      </c>
+      <c r="E151" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F151" s="8" t="inlineStr">
+        <is>
+          <t>1. Period = Last 12 months; note every KPI card and the funnel
+2. Apply Lead Source and Project
+3. Set each of the 8 filters to its "All …" option one by one (not Reset filters)</t>
+        </is>
+      </c>
+      <c r="G151" s="8" t="inlineStr">
+        <is>
+          <t>Last 12 months; filter values are picked from the page at run time</t>
+        </is>
+      </c>
+      <c r="H151" s="8" t="inlineStr">
+        <is>
+          <t>Every filter shows "All …"; every KPI card and every funnel step equal step 1</t>
+        </is>
+      </c>
+      <c r="I151" s="8" t="inlineStr">
+        <is>
+          <t>Digital Marketing + Palm Exotjca Limited (1 lead), then each filter set back to All: all 8 KPI cards and every funnel step equal the unfiltered values</t>
+        </is>
+      </c>
+      <c r="J151" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K151" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L151" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M151" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-combinations.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="8" t="inlineStr">
+        <is>
+          <t>LR-151</t>
+        </is>
+      </c>
+      <c r="B152" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C152" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="D152" s="8" t="inlineStr">
+        <is>
+          <t>Verify filter results contain no records outside the selected filter criteria</t>
+        </is>
+      </c>
+      <c r="E152" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F152" s="8" t="inlineStr">
+        <is>
+          <t>1. Period = Last 12 months
+2. Apply Lead Source, Capture Channel, Salesperson and Project values that still have leads together
+3. Click the Leads Captured count and Export the list</t>
+        </is>
+      </c>
+      <c r="G152" s="8" t="inlineStr">
+        <is>
+          <t>Last 12 months; filter values are picked from the page at run time</t>
+        </is>
+      </c>
+      <c r="H152" s="8" t="inlineStr">
+        <is>
+          <t>Every listed and exported lead has the selected Source, Channel, Salesperson and Project; list count = export rows = Leads Captured</t>
+        </is>
+      </c>
+      <c r="I152" s="8" t="inlineStr">
+        <is>
+          <t>Digital Marketing + Google Ads + CRM Administrator + Palm Exotjca Limited: 1 lead; list 1 = export 1; Source, Channel, Salesperson and Project all match (the export shows the project by its code, PEX-WATAMU)</t>
+        </is>
+      </c>
+      <c r="J152" s="8" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="K152" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L152" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M152" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-combinations.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="8" t="inlineStr">
+        <is>
+          <t>LR-152</t>
+        </is>
+      </c>
+      <c r="B153" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C153" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="D153" s="8" t="inlineStr">
+        <is>
+          <t>Verify filters work correctly when the selected combination returns exactly one lead</t>
+        </is>
+      </c>
+      <c r="E153" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F153" s="8" t="inlineStr">
+        <is>
+          <t>1. Period = Last 12 months
+2. On Source &amp; Channel find a filter value whose row shows exactly 1 lead and apply it
+3. Check the cards, funnel, Source &amp; Channel, Scorecard and the Leads Captured list</t>
+        </is>
+      </c>
+      <c r="G153" s="8" t="inlineStr">
+        <is>
+          <t>Last 12 months; filter values are picked from the page at run time</t>
+        </is>
+      </c>
+      <c r="H153" s="8" t="inlineStr">
+        <is>
+          <t>Leads Captured = 1 = funnel Captured = Source &amp; Channel Total = Scorecard Leads total; rates are only 0% or 100%; the list shows 1 lead and its export 1 row; no NaN / errors</t>
+        </is>
+      </c>
+      <c r="I153" s="8" t="inlineStr">
+        <is>
+          <t>Lead Source = Events &amp; Exhibitions: Leads Captured 1; every funnel step ≤ 1; rates 0% / 100%; list and export 1 row; Source &amp; Channel and Scorecard totals 1; Avg Time to First Contact shows — (lead not contacted)</t>
+        </is>
+      </c>
+      <c r="J153" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K153" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L153" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M153" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-combinations.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="8" t="inlineStr">
+        <is>
+          <t>LR-153</t>
+        </is>
+      </c>
+      <c r="B154" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C154" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="D154" s="8" t="inlineStr">
+        <is>
+          <t>Verify filters work correctly when no records match the selected combination</t>
+        </is>
+      </c>
+      <c r="E154" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F154" s="8" t="inlineStr">
+        <is>
+          <t>1. Period = Last 12 months; apply Lead Source = A
+2. On Source &amp; Channel find a value of another field with no leads from A and apply it
+3. Check every tab</t>
+        </is>
+      </c>
+      <c r="G154" s="8" t="inlineStr">
+        <is>
+          <t>Last 12 months; filter values are picked from the page at run time</t>
+        </is>
+      </c>
+      <c r="H154" s="8" t="inlineStr">
+        <is>
+          <t>Leads Captured, SPA Signed, Won Value and every funnel step are 0; rates show "—" or 0%; zero counts are not links; no NaN / undefined / error message; tables show no data rows</t>
+        </is>
+      </c>
+      <c r="I154" s="8" t="inlineStr">
+        <is>
+          <t>Lead Source = Referrals + Capture Channel = Bank Referral: Leads Captured, SPA Signed, Won Value and funnel all 0; rates — / 0%; no zero-count links; no NaN or error message on any tab</t>
+        </is>
+      </c>
+      <c r="J154" s="8" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K154" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L154" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M154" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-combinations.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="8" t="inlineStr">
+        <is>
+          <t>LR-154</t>
+        </is>
+      </c>
+      <c r="B155" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C155" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="D155" s="8" t="inlineStr">
+        <is>
+          <t>Verify filter values containing NULL/blank/Unspecified records are handled correctly</t>
+        </is>
+      </c>
+      <c r="E155" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F155" s="8" t="inlineStr">
+        <is>
+          <t>1. Period = Last 12 months
+2. For each field on Source &amp; Channel note the Unspecified / Unassigned row and check that field's dropdown
+3. Apply each Lead Source option in turn and add up Leads Captured
+4. Open the list for one source</t>
+        </is>
+      </c>
+      <c r="G155" s="8" t="inlineStr">
+        <is>
+          <t>Last 12 months; filter values are picked from the page at run time</t>
+        </is>
+      </c>
+      <c r="H155" s="8" t="inlineStr">
+        <is>
+          <t>No dropdown has a blank, "null" or "undefined" option; named rows + Unspecified = Total for every field; the sum over all Lead Source options = Total − Unspecified (leads without a source are never counted under a source); no listed lead has a blank Source</t>
+        </is>
+      </c>
+      <c r="I155" s="8" t="inlineStr">
+        <is>
+          <t>No blank / null options in any filter; named rows + Unspecified = Total for all 8 fields; Lead Source: sum of the 8 options 41 = 613 − 572 Unspecified; Unspecified / Unassigned cannot be selected as a filter value</t>
+        </is>
+      </c>
+      <c r="J155" s="8" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="K155" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L155" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M155" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-combinations.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="8" t="inlineStr">
+        <is>
+          <t>LR-155</t>
+        </is>
+      </c>
+      <c r="B156" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C156" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="D156" s="8" t="inlineStr">
+        <is>
+          <t>Verify filters remain consistent when switching between report tabs</t>
+        </is>
+      </c>
+      <c r="E156" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F156" s="8" t="inlineStr">
+        <is>
+          <t>1. Period = Last 12 months; apply Lead Source = A and Project = P; note every KPI card
+2. Open each tab in turn, then return to Overview &amp; Funnel</t>
+        </is>
+      </c>
+      <c r="G156" s="8" t="inlineStr">
+        <is>
+          <t>Last 12 months; filter values are picked from the page at run time</t>
+        </is>
+      </c>
+      <c r="H156" s="8" t="inlineStr">
+        <is>
+          <t>Both filters stay selected on every tab; Source &amp; Channel Total = Leads Captured; Scorecard Leads = Leads Captured and Open Now = Open Leads Now; Aging Open = Open Leads Now; KPI cards are unchanged after returning to Overview</t>
+        </is>
+      </c>
+      <c r="I156" s="8" t="inlineStr">
+        <is>
+          <t>Digital Marketing + Palm Exotjca Limited stayed selected on all 5 tabs; Source &amp; Channel Total = Scorecard Leads = Leads Captured 1; Scorecard Open Now = Aging Open Leads = Open Leads Now 0; KPI cards unchanged after the round trip</t>
+        </is>
+      </c>
+      <c r="J156" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K156" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L156" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M156" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-combinations.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="8" t="inlineStr">
+        <is>
+          <t>LR-156</t>
+        </is>
+      </c>
+      <c r="B157" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C157" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="D157" s="8" t="inlineStr">
+        <is>
+          <t>Verify filter values themselves are populated with the correct available master-data values</t>
+        </is>
+      </c>
+      <c r="E157" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F157" s="8" t="inlineStr">
+        <is>
+          <t>1. Period = Last 12 months, no filters
+2. For each of the 8 filters compare the dropdown with the options API (/reports/leads/options) and with Source &amp; Channel › Performance by &lt;that field&gt;</t>
+        </is>
+      </c>
+      <c r="G157" s="8" t="inlineStr">
+        <is>
+          <t>Last 12 months; filter values are picked from the page at run time</t>
+        </is>
+      </c>
+      <c r="H157" s="8" t="inlineStr">
+        <is>
+          <t>Dropdown = options API list in the same order; no blank or duplicate labels; every value that has leads (except Unspecified / Unassigned) can be selected</t>
+        </is>
+      </c>
+      <c r="I157" s="8" t="inlineStr">
+        <is>
+          <t>Dropdowns = options API for all 8 fields. Project lists 2 projects, but 9 project codes with leads cannot be selected (**&amp;**&amp;*&amp;**, PES-EXOT, PET, PET-AEX-001, PEX, PEX_EXOT, PRJ, PRJE, PROJ) and "QA Test Project 01" has no leads; Salesperson lists "Mahalakshmi" twice (two users, same label)</t>
+        </is>
+      </c>
+      <c r="J157" s="8" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="K157" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L157" s="17" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="M157" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-combinations.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="8" t="inlineStr">
+        <is>
+          <t>LR-157</t>
+        </is>
+      </c>
+      <c r="B158" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C158" s="8" t="inlineStr">
+        <is>
+          <t>Filter counts</t>
+        </is>
+      </c>
+      <c r="D158" s="8" t="inlineStr">
+        <is>
+          <t>Apply each filter and verify the Overview counts equal that value's row in Performance by &lt;field&gt;</t>
+        </is>
+      </c>
+      <c r="E158" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F158" s="8" t="inlineStr">
+        <is>
+          <t>1. On Source &amp; Channel › Performance by &lt;field&gt; note the row of the value to filter by
+2. Reload, set only that filter
+3. Read Leads Captured, SPA Signed, Won Value and every Lead Funnel step
+4. Repeat for every filter</t>
+        </is>
+      </c>
+      <c r="G158" s="8" t="inlineStr">
+        <is>
+          <t>Period = Last 12 months. Each of the 8 filters (Project, Lead Source, Capture Channel, Campaign, Broker, Salesperson, Prospect Type, Nationality) is applied on its own, in turn, with its busiest value that has some but not all of the leads (picked from Source &amp; Channel › Performance by &lt;field&gt; at run time)</t>
+        </is>
+      </c>
+      <c r="H158" s="8" t="inlineStr">
+        <is>
+          <t>Leads Captured = row Leads; funnel Captured / Contacted / Qualified / Opportunity / Reserved / SPA Signed = the row's columns; SPA Signed card = row SPA Signed; Won Value card = row Won Value</t>
+        </is>
+      </c>
+      <c r="I158" s="8" t="inlineStr">
+        <is>
+          <t>Values: Digital Marketing 18, Google Ads 5, Palm Exotica Campaign 2026-06 108, Palm Exotica Broker 1 15, CRM Administrator 597, Palm Exotjca Limited 555, India 8, Individual (Person) 41 (of 613). All 8: Leads Captured, every funnel step, SPA Signed and Won Value = the row (e.g. Digital Marketing 18 / 14 / 14 / 12 / 9 / 7, 7.7M USD)</t>
+        </is>
+      </c>
+      <c r="J158" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K158" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L158" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M158" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-counts.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="8" t="inlineStr">
+        <is>
+          <t>LR-158</t>
+        </is>
+      </c>
+      <c r="B159" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C159" s="8" t="inlineStr">
+        <is>
+          <t>Filter counts</t>
+        </is>
+      </c>
+      <c r="D159" s="8" t="inlineStr">
+        <is>
+          <t>Apply each filter and verify the rate cards are recalculated from the filtered counts</t>
+        </is>
+      </c>
+      <c r="E159" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F159" s="8" t="inlineStr">
+        <is>
+          <t>1. On Source &amp; Channel › Performance by &lt;field&gt; note the row of the value to filter by
+2. Reload, set only that filter
+3. Read Contact Rate, Qualification Rate, Opportunity Conversion, the SPA Signed Win rate and the funnel %
+4. Repeat for every filter</t>
+        </is>
+      </c>
+      <c r="G159" s="8" t="inlineStr">
+        <is>
+          <t>Period = Last 12 months. Each of the 8 filters (Project, Lead Source, Capture Channel, Campaign, Broker, Salesperson, Prospect Type, Nationality) is applied on its own, in turn, with its busiest value that has some but not all of the leads (picked from Source &amp; Channel › Performance by &lt;field&gt; at run time)</t>
+        </is>
+      </c>
+      <c r="H159" s="8" t="inlineStr">
+        <is>
+          <t>Each rate = its funnel count ÷ Leads Captured = the funnel % = the row's Contact % / Qual. % / Conv. % / Win % (±0.1)</t>
+        </is>
+      </c>
+      <c r="I159" s="8" t="inlineStr">
+        <is>
+          <t>Values: Digital Marketing 18, Google Ads 5, Palm Exotica Campaign 2026-06 108, Palm Exotica Broker 1 15, CRM Administrator 597, Palm Exotjca Limited 555, India 8, Individual (Person) 41 (of 613). All 8: Contact, Qualification, Opportunity and Win rates = count ÷ Leads Captured = funnel % = row %</t>
+        </is>
+      </c>
+      <c r="J159" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K159" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L159" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M159" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-counts.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="8" t="inlineStr">
+        <is>
+          <t>LR-159</t>
+        </is>
+      </c>
+      <c r="B160" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C160" s="8" t="inlineStr">
+        <is>
+          <t>Filter counts</t>
+        </is>
+      </c>
+      <c r="D160" s="8" t="inlineStr">
+        <is>
+          <t>Apply each filter and verify each count card opens a list with that many leads, all matching the filter</t>
+        </is>
+      </c>
+      <c r="E160" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F160" s="8" t="inlineStr">
+        <is>
+          <t>1. On Source &amp; Channel › Performance by &lt;field&gt; note the row of the value to filter by
+2. Reload, set only that filter
+3. Click Leads Captured (and Export), SPA Signed and Open Leads Now
+4. Repeat for every filter</t>
+        </is>
+      </c>
+      <c r="G160" s="8" t="inlineStr">
+        <is>
+          <t>Period = Last 12 months. Each of the 8 filters (Project, Lead Source, Capture Channel, Campaign, Broker, Salesperson, Prospect Type, Nationality) is applied on its own, in turn, with its busiest value that has some but not all of the leads (picked from Source &amp; Channel › Performance by &lt;field&gt; at run time)</t>
+        </is>
+      </c>
+      <c r="H160" s="8" t="inlineStr">
+        <is>
+          <t>Each list header, rows and export = the card count; every listed lead has the selected value (Source, Channel, Salesperson, Project are checked on the list / export)</t>
+        </is>
+      </c>
+      <c r="I160" s="8" t="inlineStr">
+        <is>
+          <t>All 8 lists = card counts (e.g. CRM Administrator: Leads Captured 597, SPA Signed 76, Open Leads Now 354); no lead outside the filter on Source, Channel, Salesperson, Project</t>
+        </is>
+      </c>
+      <c r="J160" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K160" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L160" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M160" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-counts.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="8" t="inlineStr">
+        <is>
+          <t>LR-160</t>
+        </is>
+      </c>
+      <c r="B161" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C161" s="8" t="inlineStr">
+        <is>
+          <t>Filter counts</t>
+        </is>
+      </c>
+      <c r="D161" s="8" t="inlineStr">
+        <is>
+          <t>Apply each filter and verify Data Completeness and the 12-Month Trend follow the filter</t>
+        </is>
+      </c>
+      <c r="E161" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F161" s="8" t="inlineStr">
+        <is>
+          <t>1. On Source &amp; Channel › Performance by &lt;field&gt; note the row of the value to filter by
+2. Reload, set only that filter
+3. Read Data Completeness and the 12-Month Trend
+4. Repeat for every filter</t>
+        </is>
+      </c>
+      <c r="G161" s="8" t="inlineStr">
+        <is>
+          <t>Period = Last 12 months. Each of the 8 filters (Project, Lead Source, Capture Channel, Campaign, Broker, Salesperson, Prospect Type, Nationality) is applied on its own, in turn, with its busiest value that has some but not all of the leads (picked from Source &amp; Channel › Performance by &lt;field&gt; at run time)</t>
+        </is>
+      </c>
+      <c r="H161" s="8" t="inlineStr">
+        <is>
+          <t>Every Data Completeness row shows "x / &lt;filtered Leads Captured&gt;"; the 12 months add up to the filtered Leads Captured</t>
+        </is>
+      </c>
+      <c r="I161" s="8" t="inlineStr">
+        <is>
+          <t>All 8: every Data Completeness row totals the filtered Leads Captured; 12-Month Trend adds up to it</t>
+        </is>
+      </c>
+      <c r="J161" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K161" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L161" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M161" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-counts.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="8" t="inlineStr">
+        <is>
+          <t>LR-161</t>
+        </is>
+      </c>
+      <c r="B162" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>Filter counts</t>
+        </is>
+      </c>
+      <c r="D162" s="8" t="inlineStr">
+        <is>
+          <t>Apply each filter and verify every Source &amp; Channel grouping totals to the filtered counts</t>
+        </is>
+      </c>
+      <c r="E162" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F162" s="8" t="inlineStr">
+        <is>
+          <t>1. On Source &amp; Channel › Performance by &lt;field&gt; note the row of the value to filter by
+2. Reload, set only that filter
+3. Open Source &amp; Channel and switch through all 8 groupings
+4. Repeat for every filter</t>
+        </is>
+      </c>
+      <c r="G162" s="8" t="inlineStr">
+        <is>
+          <t>Period = Last 12 months. Each of the 8 filters (Project, Lead Source, Capture Channel, Campaign, Broker, Salesperson, Prospect Type, Nationality) is applied on its own, in turn, with its busiest value that has some but not all of the leads (picked from Source &amp; Channel › Performance by &lt;field&gt; at run time)</t>
+        </is>
+      </c>
+      <c r="H162" s="8" t="inlineStr">
+        <is>
+          <t>For every grouping: Total Leads = Leads Captured and Total Contacted / Qualified / Opportunity / Reserved / SPA Signed = the funnel; the filtered field lists only the selected value</t>
+        </is>
+      </c>
+      <c r="I162" s="8" t="inlineStr">
+        <is>
+          <t>All 8 filters × 8 groupings: Total Leads = Leads Captured and Total Contacted…SPA Signed = funnel; filtered field lists only the selected value</t>
+        </is>
+      </c>
+      <c r="J162" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K162" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L162" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M162" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-counts.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="8" t="inlineStr">
+        <is>
+          <t>LR-162</t>
+        </is>
+      </c>
+      <c r="B163" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C163" s="8" t="inlineStr">
+        <is>
+          <t>Filter counts</t>
+        </is>
+      </c>
+      <c r="D163" s="8" t="inlineStr">
+        <is>
+          <t>Apply each filter and verify the Aging &amp; Follow-up counts</t>
+        </is>
+      </c>
+      <c r="E163" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F163" s="8" t="inlineStr">
+        <is>
+          <t>1. On Source &amp; Channel › Performance by &lt;field&gt; note the row of the value to filter by
+2. Reload, set only that filter
+3. Note Open Leads Now; open Aging &amp; Follow-up
+4. Repeat for every filter</t>
+        </is>
+      </c>
+      <c r="G163" s="8" t="inlineStr">
+        <is>
+          <t>Period = Last 12 months. Each of the 8 filters (Project, Lead Source, Capture Channel, Campaign, Broker, Salesperson, Prospect Type, Nationality) is applied on its own, in turn, with its busiest value that has some but not all of the leads (picked from Source &amp; Channel › Performance by &lt;field&gt; at run time)</t>
+        </is>
+      </c>
+      <c r="H163" s="8" t="inlineStr">
+        <is>
+          <t>Open Leads = Open Leads Now; Never Contacted and Idle Over 30 Days ≤ Open Leads; Idle Time and Lead Age buckets add up to Open Leads; Open Leads by Salesperson Open / Never Contacted / Overdue columns = the cards</t>
+        </is>
+      </c>
+      <c r="I163" s="8" t="inlineStr">
+        <is>
+          <t>All 8: Aging Open Leads = Open Leads Now (e.g. Campaign 2026-06: 65), buckets and Open Leads by Salesperson add up to it; Never Contacted / Idle ≤ Open</t>
+        </is>
+      </c>
+      <c r="J163" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K163" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L163" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M163" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-counts.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="8" t="inlineStr">
+        <is>
+          <t>LR-163</t>
+        </is>
+      </c>
+      <c r="B164" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C164" s="8" t="inlineStr">
+        <is>
+          <t>Filter counts</t>
+        </is>
+      </c>
+      <c r="D164" s="8" t="inlineStr">
+        <is>
+          <t>Apply each filter and verify the Qualification &amp; Conversion counts</t>
+        </is>
+      </c>
+      <c r="E164" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F164" s="8" t="inlineStr">
+        <is>
+          <t>1. On Source &amp; Channel › Performance by &lt;field&gt; note the row of the value to filter by
+2. Reload, set only that filter
+3. Note the Lost total on Source &amp; Channel; open Qualification &amp; Conversion; click View lost leads
+4. Repeat for every filter</t>
+        </is>
+      </c>
+      <c r="G164" s="8" t="inlineStr">
+        <is>
+          <t>Period = Last 12 months. Each of the 8 filters (Project, Lead Source, Capture Channel, Campaign, Broker, Salesperson, Prospect Type, Nationality) is applied on its own, in turn, with its busiest value that has some but not all of the leads (picked from Source &amp; Channel › Performance by &lt;field&gt; at run time)</t>
+        </is>
+      </c>
+      <c r="H164" s="8" t="inlineStr">
+        <is>
+          <t>Conversion by Lead Rating, Conversion by Lead Score and Where the Leads Are Now each add up to Leads Captured; Lost Reasons add up to Lost; the lost-leads list has that many leads</t>
+        </is>
+      </c>
+      <c r="I164" s="8" t="inlineStr">
+        <is>
+          <t>All 8: Lead Rating, Lead Score and Where the Leads Are Now add up to Leads Captured; Lost Reasons = Lost (e.g. CRM Administrator 127 = 127) and the lost list matches</t>
+        </is>
+      </c>
+      <c r="J164" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K164" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L164" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M164" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-counts.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="8" t="inlineStr">
+        <is>
+          <t>LR-164</t>
+        </is>
+      </c>
+      <c r="B165" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C165" s="8" t="inlineStr">
+        <is>
+          <t>Filter counts</t>
+        </is>
+      </c>
+      <c r="D165" s="8" t="inlineStr">
+        <is>
+          <t>Apply each filter and verify the Salesperson Scorecard totals</t>
+        </is>
+      </c>
+      <c r="E165" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F165" s="8" t="inlineStr">
+        <is>
+          <t>1. On Source &amp; Channel › Performance by &lt;field&gt; note the row of the value to filter by
+2. Reload, set only that filter
+3. Note the funnel and cards; open Aging &amp; Follow-up, then Salesperson Scorecard
+4. Repeat for every filter</t>
+        </is>
+      </c>
+      <c r="G165" s="8" t="inlineStr">
+        <is>
+          <t>Period = Last 12 months. Each of the 8 filters (Project, Lead Source, Capture Channel, Campaign, Broker, Salesperson, Prospect Type, Nationality) is applied on its own, in turn, with its busiest value that has some but not all of the leads (picked from Source &amp; Channel › Performance by &lt;field&gt; at run time)</t>
+        </is>
+      </c>
+      <c r="H165" s="8" t="inlineStr">
+        <is>
+          <t>Scorecard Leads = Leads Captured; Contacted / Qualified / Opportunity = funnel; SPA Signed = card; Open Now = Open Leads Now; each salesperson's Open Now = their Aging Open</t>
+        </is>
+      </c>
+      <c r="I165" s="8" t="inlineStr">
+        <is>
+          <t>All 8: Scorecard Leads, Contacted, Qualified, Opportunity, SPA Signed and Open Now totals = the cards / funnel; each salesperson's Open Now = Aging Open</t>
+        </is>
+      </c>
+      <c r="J165" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K165" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L165" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M165" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-counts.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="8" t="inlineStr">
+        <is>
+          <t>LR-165</t>
+        </is>
+      </c>
+      <c r="B166" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C166" s="8" t="inlineStr">
+        <is>
+          <t>Filter counts</t>
+        </is>
+      </c>
+      <c r="D166" s="8" t="inlineStr">
+        <is>
+          <t>Apply every value of each filter in turn and verify the filtered counts add up to the unfiltered total</t>
+        </is>
+      </c>
+      <c r="E166" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F166" s="8" t="inlineStr">
+        <is>
+          <t>1. On Source &amp; Channel note each field's Total and Unspecified / Unassigned row
+2. For each filter, select every option in turn and read Leads Captured
+3. Add up the counts per filter</t>
+        </is>
+      </c>
+      <c r="G166" s="8" t="inlineStr">
+        <is>
+          <t>Period = Last 12 months; every option of all 8 filters</t>
+        </is>
+      </c>
+      <c r="H166" s="8" t="inlineStr">
+        <is>
+          <t>For every filter: sum of Leads Captured over its options = Total − Unspecified (every lead with a value is counted under exactly one option)</t>
+        </is>
+      </c>
+      <c r="I166" s="8" t="inlineStr">
+        <is>
+          <t>Lead Source 41 = 613 − 572; Capture Channel 26; Campaign 568; Broker 149; Salesperson 611; Nationality 34; Prospect Type 44 — all add up. Project: 555 + 0 = 555 but Total − Unspecified = 564: 9 leads have project codes not in the Project filter (see LR-156)</t>
+        </is>
+      </c>
+      <c r="J166" s="8" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="K166" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L166" s="17" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="M166" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-counts.spec.ts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="8" t="inlineStr">
+        <is>
+          <t>LR-166</t>
+        </is>
+      </c>
+      <c r="B167" s="8" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="C167" s="8" t="inlineStr">
+        <is>
+          <t>Filter counts</t>
+        </is>
+      </c>
+      <c r="D167" s="8" t="inlineStr">
+        <is>
+          <t>Apply each filter with the period "This month" and verify the counts equal that value's row</t>
+        </is>
+      </c>
+      <c r="E167" s="8" t="inlineStr">
+        <is>
+          <t>Logged in as CRM Administrator; Lead Reports open (https://qa-crm.asquareab.com/reports/leads)</t>
+        </is>
+      </c>
+      <c r="F167" s="8" t="inlineStr">
+        <is>
+          <t>1. Period = This month; on Source &amp; Channel note the row of the value to filter by
+2. Reload on This month, set only that filter
+3. Read Leads Captured, SPA Signed, Won Value and the funnel
+4. Repeat for every filter</t>
+        </is>
+      </c>
+      <c r="G167" s="8" t="inlineStr">
+        <is>
+          <t>Period = This month; values picked from This month's Performance by &lt;field&gt;</t>
+        </is>
+      </c>
+      <c r="H167" s="8" t="inlineStr">
+        <is>
+          <t>Same as LR-157 for This month: cards and funnel = the value's row; filters with no value this month are skipped</t>
+        </is>
+      </c>
+      <c r="I167" s="8" t="inlineStr">
+        <is>
+          <t>This month (16 leads): Digital Marketing 6, qabroker 3, CRM Administrator 11, Palm Exotjca Limited 1, Canada 2, Individual (Person) 14 — cards and funnel = the row; Capture Channel and Campaign had no value this month (skipped)</t>
+        </is>
+      </c>
+      <c r="J167" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K167" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L167" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M167" s="8" t="inlineStr">
+        <is>
+          <t>Executed 15-Oct-2026 (automated: tests/lead-reports/filter-counts.spec.ts)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M147"/>
+  <autoFilter ref="A1:M167"/>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L2:L167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,Pass,Fail,Blocked,Not Applicable"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>